<commit_message>
Adiciona aba com o laudo SGS Geosol 2024 (4 amostras de superfície)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017WeXEcDzNZfvUSeTFqUMWA
</commit_message>
<xml_diff>
--- a/uranio_diques_estatistica.xlsx
+++ b/uranio_diques_estatistica.xlsx
@@ -16,6 +16,7 @@
     <sheet name="Correlação" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="Dendrograma" sheetId="7" state="visible" r:id="rId9"/>
     <sheet name="Comparação artigo" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="Laudo SGS 2024" sheetId="9" state="visible" r:id="rId11"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -49,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="281">
   <si>
     <t xml:space="preserve">Conclusões integradas (estatística das Tabelas 1–2 + matriz de correlação e dendrograma)</t>
   </si>
@@ -688,6 +689,210 @@
   </si>
   <si>
     <t xml:space="preserve">Erro de digitação no texto: a Tabela 3 traz 0,4322.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Laudo SGS Geosol GQ2407332 (emitido em 12/08/2024) – 4 amostras de superfície, Pedreira Genaro, Catanduvas de Fora, Carambeí/PR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fusão com metaborato de lítio; ICP-OES (maiores) e ICP-MS (traços). Óxidos e LOI em %, demais em ppm. Valores transcritos em azul; '&lt;LD' deixado em branco.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analito</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AM 01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AM 02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AM 03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AM 04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REP AM 04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BRANCO_PREP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MgO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P2O5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ce</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Co</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Er</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ga</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ho</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ni</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Th</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PARÂMETROS CALCULADOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Soma óxidos + LOI (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U3O8 (ppm) = U × 1,1792</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ThO2 (ppm) = Th × 1,1379</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Th/U</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Índice agpaítico (Na+K)/Al molar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ASI Al/(Ca+Na+K) molar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10⁴·Ga/Al (tipo A &gt; 2,6)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zr+Nb+Ce+Y (tipo A &gt; 350 ppm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rb/Sr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eu/Eu* (condrito Sun &amp; McDonough 1989)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(La/Yb)N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ra-226 estimado (Bq/kg) = U × 12,35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Th-232 (Bq/kg) = Th × 4,06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K-40 (Bq/kg) = K2O × 0,8301 × 313</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Índice I (Ra/300 + Th/200 + K/3000)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eu de AM 02 &lt; LD (0,05 ppm): Eu/Eu* não calculado; nas demais, Eu está no LD, então Eu/Eu* é valor máximo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ra-226 supõe equilíbrio secular com U-238, hipótese frágil numa rocha em que ~70% do U é solúvel (Tabela 1, 1988). Medir por espectrometria gama.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Índice I (Diretiva 2013/59/Euratom, Anexo VIII): triagem para material de construção; I ≤ 1 em uso de massa. Referência europeia, não norma brasileira.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Soma de óxidos fora de 98,5–101,5% em AM 02, AM 03 e AM 04; réplica de AM 04 difere 2 pontos em SiO2. Os óxidos maiores são pouco precisos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMPARAÇÃO DO U3O8 COM 1988 (superfície CV)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mediana U3O8 – 2024 (4 amostras)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mediana U3O8 – 1988 superfície (CV)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faixa 1988 superfície (mín–máx)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faixa 1988 granito subsuperfície (mín–máx)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Limiar de anomalia do granito (média+2DP)</t>
   </si>
 </sst>
 </file>
@@ -890,7 +1095,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="50">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1080,6 +1285,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="173" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -6876,4 +7089,1515 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G79"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="0" width="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="22" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="48" t="s">
+        <v>215</v>
+      </c>
+      <c r="B4" s="48" t="s">
+        <v>216</v>
+      </c>
+      <c r="C4" s="48" t="s">
+        <v>217</v>
+      </c>
+      <c r="D4" s="48" t="s">
+        <v>218</v>
+      </c>
+      <c r="E4" s="48" t="s">
+        <v>219</v>
+      </c>
+      <c r="F4" s="48" t="s">
+        <v>220</v>
+      </c>
+      <c r="G4" s="48" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="39" t="s">
+        <v>141</v>
+      </c>
+      <c r="B5" s="43" t="n">
+        <v>11.85</v>
+      </c>
+      <c r="C5" s="43" t="n">
+        <v>12.57</v>
+      </c>
+      <c r="D5" s="43" t="n">
+        <v>11.59</v>
+      </c>
+      <c r="E5" s="43" t="n">
+        <v>12.62</v>
+      </c>
+      <c r="F5" s="43" t="n">
+        <v>12.22</v>
+      </c>
+      <c r="G5" s="43" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="39" t="s">
+        <v>144</v>
+      </c>
+      <c r="B6" s="43" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="C6" s="43" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="D6" s="43" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="E6" s="43" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F6" s="43" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="G6" s="43" t="n">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="39" t="s">
+        <v>142</v>
+      </c>
+      <c r="B7" s="43" t="n">
+        <v>2.59</v>
+      </c>
+      <c r="C7" s="43" t="n">
+        <v>2.76</v>
+      </c>
+      <c r="D7" s="43" t="n">
+        <v>2.37</v>
+      </c>
+      <c r="E7" s="43" t="n">
+        <v>1.95</v>
+      </c>
+      <c r="F7" s="43" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="G7" s="43" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="39" t="s">
+        <v>146</v>
+      </c>
+      <c r="B8" s="43" t="n">
+        <v>4.08</v>
+      </c>
+      <c r="C8" s="43" t="n">
+        <v>3.61</v>
+      </c>
+      <c r="D8" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="E8" s="43" t="n">
+        <v>4.36</v>
+      </c>
+      <c r="F8" s="43" t="n">
+        <v>4.21</v>
+      </c>
+      <c r="G8" s="43" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="39" t="s">
+        <v>222</v>
+      </c>
+      <c r="B9" s="43" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C9" s="43" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="D9" s="43" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="E9" s="43" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F9" s="43" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="G9" s="43" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="39" t="s">
+        <v>147</v>
+      </c>
+      <c r="B10" s="43" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="C10" s="43" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="D10" s="43" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="E10" s="43" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F10" s="43" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="G10" s="43"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="39" t="s">
+        <v>145</v>
+      </c>
+      <c r="B11" s="43" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="C11" s="43" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="D11" s="43" t="n">
+        <v>3.94</v>
+      </c>
+      <c r="E11" s="43" t="n">
+        <v>4.06</v>
+      </c>
+      <c r="F11" s="43" t="n">
+        <v>3.95</v>
+      </c>
+      <c r="G11" s="43" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="39" t="s">
+        <v>223</v>
+      </c>
+      <c r="B12" s="43"/>
+      <c r="C12" s="43"/>
+      <c r="D12" s="43" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="E12" s="43"/>
+      <c r="F12" s="43"/>
+      <c r="G12" s="43"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="39" t="s">
+        <v>139</v>
+      </c>
+      <c r="B13" s="43" t="n">
+        <v>76.27</v>
+      </c>
+      <c r="C13" s="43" t="n">
+        <v>71.91</v>
+      </c>
+      <c r="D13" s="43" t="n">
+        <v>71.95</v>
+      </c>
+      <c r="E13" s="43" t="n">
+        <v>78.52</v>
+      </c>
+      <c r="F13" s="43" t="n">
+        <v>76.55</v>
+      </c>
+      <c r="G13" s="43"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="39" t="s">
+        <v>140</v>
+      </c>
+      <c r="B14" s="43" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C14" s="43" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="D14" s="43" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="E14" s="43" t="n">
+        <v>0.07</v>
+      </c>
+      <c r="F14" s="43" t="n">
+        <v>0.07</v>
+      </c>
+      <c r="G14" s="43"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="39" t="s">
+        <v>224</v>
+      </c>
+      <c r="B15" s="43" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="C15" s="43" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="D15" s="43" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="E15" s="43" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="F15" s="43" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="G15" s="43" t="n">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="39" t="s">
+        <v>225</v>
+      </c>
+      <c r="B16" s="43" t="n">
+        <v>37</v>
+      </c>
+      <c r="C16" s="43" t="n">
+        <v>55</v>
+      </c>
+      <c r="D16" s="43" t="n">
+        <v>26</v>
+      </c>
+      <c r="E16" s="43" t="n">
+        <v>22</v>
+      </c>
+      <c r="F16" s="43" t="n">
+        <v>27</v>
+      </c>
+      <c r="G16" s="43" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="39" t="s">
+        <v>226</v>
+      </c>
+      <c r="B17" s="43" t="n">
+        <v>14</v>
+      </c>
+      <c r="C17" s="43" t="n">
+        <v>15</v>
+      </c>
+      <c r="D17" s="43" t="n">
+        <v>14</v>
+      </c>
+      <c r="E17" s="43" t="n">
+        <v>10</v>
+      </c>
+      <c r="F17" s="43" t="n">
+        <v>10</v>
+      </c>
+      <c r="G17" s="43"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="39" t="s">
+        <v>227</v>
+      </c>
+      <c r="B18" s="43" t="n">
+        <v>268</v>
+      </c>
+      <c r="C18" s="43" t="n">
+        <v>254</v>
+      </c>
+      <c r="D18" s="43" t="n">
+        <v>265</v>
+      </c>
+      <c r="E18" s="43" t="n">
+        <v>203</v>
+      </c>
+      <c r="F18" s="43" t="n">
+        <v>201</v>
+      </c>
+      <c r="G18" s="43" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="39" t="s">
+        <v>151</v>
+      </c>
+      <c r="B19" s="43" t="n">
+        <v>272</v>
+      </c>
+      <c r="C19" s="43" t="n">
+        <v>208</v>
+      </c>
+      <c r="D19" s="43" t="n">
+        <v>270</v>
+      </c>
+      <c r="E19" s="43" t="n">
+        <v>243</v>
+      </c>
+      <c r="F19" s="43" t="n">
+        <v>249</v>
+      </c>
+      <c r="G19" s="43"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="39" t="s">
+        <v>228</v>
+      </c>
+      <c r="B20" s="43" t="n">
+        <v>9</v>
+      </c>
+      <c r="C20" s="43" t="n">
+        <v>48</v>
+      </c>
+      <c r="D20" s="43" t="n">
+        <v>95</v>
+      </c>
+      <c r="E20" s="43" t="n">
+        <v>42</v>
+      </c>
+      <c r="F20" s="43" t="n">
+        <v>38</v>
+      </c>
+      <c r="G20" s="43" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="39" t="s">
+        <v>229</v>
+      </c>
+      <c r="B21" s="43" t="n">
+        <v>77.9</v>
+      </c>
+      <c r="C21" s="43" t="n">
+        <v>49.3</v>
+      </c>
+      <c r="D21" s="43" t="n">
+        <v>67.7</v>
+      </c>
+      <c r="E21" s="43" t="n">
+        <v>95.5</v>
+      </c>
+      <c r="F21" s="43" t="n">
+        <v>92.3</v>
+      </c>
+      <c r="G21" s="43" t="n">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="39" t="s">
+        <v>230</v>
+      </c>
+      <c r="B22" s="43"/>
+      <c r="C22" s="43"/>
+      <c r="D22" s="43" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E22" s="43" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F22" s="43" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G22" s="43" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="39" t="s">
+        <v>231</v>
+      </c>
+      <c r="B23" s="43" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="C23" s="43" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="D23" s="43" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="E23" s="43" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="F23" s="43" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="G23" s="43" t="n">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="39" t="s">
+        <v>232</v>
+      </c>
+      <c r="B24" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="C24" s="43"/>
+      <c r="D24" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="E24" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="F24" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="G24" s="43"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="39" t="s">
+        <v>233</v>
+      </c>
+      <c r="B25" s="43" t="n">
+        <v>32.08</v>
+      </c>
+      <c r="C25" s="43" t="n">
+        <v>42.74</v>
+      </c>
+      <c r="D25" s="43" t="n">
+        <v>39.25</v>
+      </c>
+      <c r="E25" s="43" t="n">
+        <v>22.85</v>
+      </c>
+      <c r="F25" s="43" t="n">
+        <v>22.89</v>
+      </c>
+      <c r="G25" s="43" t="n">
+        <v>0.14</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="39" t="s">
+        <v>234</v>
+      </c>
+      <c r="B26" s="43" t="n">
+        <v>21.96</v>
+      </c>
+      <c r="C26" s="43" t="n">
+        <v>28.55</v>
+      </c>
+      <c r="D26" s="43" t="n">
+        <v>25.95</v>
+      </c>
+      <c r="E26" s="43" t="n">
+        <v>14.08</v>
+      </c>
+      <c r="F26" s="43" t="n">
+        <v>14.22</v>
+      </c>
+      <c r="G26" s="43" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="39" t="s">
+        <v>235</v>
+      </c>
+      <c r="B27" s="43" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C27" s="43"/>
+      <c r="D27" s="43" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E27" s="43" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="F27" s="43" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="G27" s="43"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="39" t="s">
+        <v>236</v>
+      </c>
+      <c r="B28" s="43" t="n">
+        <v>36.8</v>
+      </c>
+      <c r="C28" s="43" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="D28" s="43" t="n">
+        <v>36</v>
+      </c>
+      <c r="E28" s="43" t="n">
+        <v>39.8</v>
+      </c>
+      <c r="F28" s="43" t="n">
+        <v>39.2</v>
+      </c>
+      <c r="G28" s="43"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="39" t="s">
+        <v>237</v>
+      </c>
+      <c r="B29" s="43" t="n">
+        <v>20.33</v>
+      </c>
+      <c r="C29" s="43" t="n">
+        <v>22.94</v>
+      </c>
+      <c r="D29" s="43" t="n">
+        <v>21.93</v>
+      </c>
+      <c r="E29" s="43" t="n">
+        <v>18.39</v>
+      </c>
+      <c r="F29" s="43" t="n">
+        <v>17.98</v>
+      </c>
+      <c r="G29" s="43" t="n">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="39" t="s">
+        <v>238</v>
+      </c>
+      <c r="B30" s="43" t="n">
+        <v>12</v>
+      </c>
+      <c r="C30" s="43" t="n">
+        <v>14.17</v>
+      </c>
+      <c r="D30" s="43" t="n">
+        <v>12.07</v>
+      </c>
+      <c r="E30" s="43" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="F30" s="43" t="n">
+        <v>12.97</v>
+      </c>
+      <c r="G30" s="43" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="39" t="s">
+        <v>239</v>
+      </c>
+      <c r="B31" s="43" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="C31" s="43" t="n">
+        <v>9.01</v>
+      </c>
+      <c r="D31" s="43" t="n">
+        <v>8.16</v>
+      </c>
+      <c r="E31" s="43" t="n">
+        <v>4.69</v>
+      </c>
+      <c r="F31" s="43" t="n">
+        <v>4.58</v>
+      </c>
+      <c r="G31" s="43"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="39" t="s">
+        <v>240</v>
+      </c>
+      <c r="B32" s="43" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="C32" s="43" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="D32" s="43" t="n">
+        <v>33.8</v>
+      </c>
+      <c r="E32" s="43" t="n">
+        <v>49.3</v>
+      </c>
+      <c r="F32" s="43" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="G32" s="43" t="n">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="39" t="s">
+        <v>241</v>
+      </c>
+      <c r="B33" s="43" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="C33" s="43" t="n">
+        <v>2.99</v>
+      </c>
+      <c r="D33" s="43" t="n">
+        <v>2.86</v>
+      </c>
+      <c r="E33" s="43" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="F33" s="43" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="G33" s="43"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="39" t="s">
+        <v>242</v>
+      </c>
+      <c r="B34" s="43"/>
+      <c r="C34" s="43" t="n">
+        <v>2</v>
+      </c>
+      <c r="D34" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="E34" s="43" t="n">
+        <v>2</v>
+      </c>
+      <c r="F34" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="G34" s="43" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="39" t="s">
+        <v>149</v>
+      </c>
+      <c r="B35" s="43" t="n">
+        <v>85.03</v>
+      </c>
+      <c r="C35" s="43" t="n">
+        <v>71.24</v>
+      </c>
+      <c r="D35" s="43" t="n">
+        <v>64.89</v>
+      </c>
+      <c r="E35" s="43" t="n">
+        <v>86.16</v>
+      </c>
+      <c r="F35" s="43" t="n">
+        <v>83.98</v>
+      </c>
+      <c r="G35" s="43"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="39" t="s">
+        <v>243</v>
+      </c>
+      <c r="B36" s="43" t="n">
+        <v>37.7</v>
+      </c>
+      <c r="C36" s="43" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="D36" s="43" t="n">
+        <v>33.7</v>
+      </c>
+      <c r="E36" s="43" t="n">
+        <v>46.2</v>
+      </c>
+      <c r="F36" s="43" t="n">
+        <v>45.1</v>
+      </c>
+      <c r="G36" s="43" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="39" t="s">
+        <v>244</v>
+      </c>
+      <c r="B37" s="43" t="n">
+        <v>8</v>
+      </c>
+      <c r="C37" s="43" t="n">
+        <v>8</v>
+      </c>
+      <c r="D37" s="43" t="n">
+        <v>21</v>
+      </c>
+      <c r="E37" s="43" t="n">
+        <v>9</v>
+      </c>
+      <c r="F37" s="43" t="n">
+        <v>17</v>
+      </c>
+      <c r="G37" s="43" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="39" t="s">
+        <v>245</v>
+      </c>
+      <c r="B38" s="43" t="n">
+        <v>9.84</v>
+      </c>
+      <c r="C38" s="43" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="D38" s="43" t="n">
+        <v>8.49</v>
+      </c>
+      <c r="E38" s="43" t="n">
+        <v>12.39</v>
+      </c>
+      <c r="F38" s="43" t="n">
+        <v>11.95</v>
+      </c>
+      <c r="G38" s="43" t="n">
+        <v>0.26</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="39" t="s">
+        <v>246</v>
+      </c>
+      <c r="B39" s="43" t="n">
+        <v>331.1</v>
+      </c>
+      <c r="C39" s="43" t="n">
+        <v>324.2</v>
+      </c>
+      <c r="D39" s="43" t="n">
+        <v>329.4</v>
+      </c>
+      <c r="E39" s="43" t="n">
+        <v>382.8</v>
+      </c>
+      <c r="F39" s="43" t="n">
+        <v>371.5</v>
+      </c>
+      <c r="G39" s="43" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="39" t="s">
+        <v>247</v>
+      </c>
+      <c r="B40" s="43" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="C40" s="43" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="D40" s="43" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="E40" s="43" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="F40" s="43" t="n">
+        <v>15</v>
+      </c>
+      <c r="G40" s="43" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="39" t="s">
+        <v>148</v>
+      </c>
+      <c r="B41" s="43" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="C41" s="43" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="D41" s="43" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="E41" s="43" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="F41" s="43" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="G41" s="43" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="39" t="s">
+        <v>248</v>
+      </c>
+      <c r="B42" s="43" t="n">
+        <v>3.74</v>
+      </c>
+      <c r="C42" s="43" t="n">
+        <v>5.69</v>
+      </c>
+      <c r="D42" s="43" t="n">
+        <v>3.04</v>
+      </c>
+      <c r="E42" s="43" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="F42" s="43" t="n">
+        <v>4.41</v>
+      </c>
+      <c r="G42" s="43"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="39" t="s">
+        <v>249</v>
+      </c>
+      <c r="B43" s="43" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="C43" s="43" t="n">
+        <v>5.38</v>
+      </c>
+      <c r="D43" s="43" t="n">
+        <v>5.04</v>
+      </c>
+      <c r="E43" s="43" t="n">
+        <v>3.43</v>
+      </c>
+      <c r="F43" s="43" t="n">
+        <v>3.33</v>
+      </c>
+      <c r="G43" s="43"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="39" t="s">
+        <v>250</v>
+      </c>
+      <c r="B44" s="43" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="C44" s="43" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="D44" s="43" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="E44" s="43" t="n">
+        <v>31.8</v>
+      </c>
+      <c r="F44" s="43" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="G44" s="43" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="39" t="s">
+        <v>251</v>
+      </c>
+      <c r="B45" s="43" t="n">
+        <v>3.16</v>
+      </c>
+      <c r="C45" s="43" t="n">
+        <v>3.89</v>
+      </c>
+      <c r="D45" s="43" t="n">
+        <v>3.66</v>
+      </c>
+      <c r="E45" s="43" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="F45" s="43" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="G45" s="43"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="39" t="s">
+        <v>252</v>
+      </c>
+      <c r="B46" s="43" t="n">
+        <v>8.14</v>
+      </c>
+      <c r="C46" s="43" t="n">
+        <v>15.38</v>
+      </c>
+      <c r="D46" s="43" t="n">
+        <v>7.69</v>
+      </c>
+      <c r="E46" s="43" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="F46" s="43" t="n">
+        <v>8.7</v>
+      </c>
+      <c r="G46" s="43" t="n">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="39" t="s">
+        <v>253</v>
+      </c>
+      <c r="B47" s="43" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="C47" s="43" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="D47" s="43" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="E47" s="43" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F47" s="43" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G47" s="43" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="39" t="s">
+        <v>150</v>
+      </c>
+      <c r="B48" s="43" t="n">
+        <v>201.44</v>
+      </c>
+      <c r="C48" s="43" t="n">
+        <v>259.19</v>
+      </c>
+      <c r="D48" s="43" t="n">
+        <v>252.8</v>
+      </c>
+      <c r="E48" s="43" t="n">
+        <v>170.21</v>
+      </c>
+      <c r="F48" s="43" t="n">
+        <v>167.87</v>
+      </c>
+      <c r="G48" s="43" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="39" t="s">
+        <v>254</v>
+      </c>
+      <c r="B49" s="43" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="C49" s="43" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="D49" s="43" t="n">
+        <v>23.1</v>
+      </c>
+      <c r="E49" s="43" t="n">
+        <v>13</v>
+      </c>
+      <c r="F49" s="43" t="n">
+        <v>13</v>
+      </c>
+      <c r="G49" s="43"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="2" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="23" t="s">
+        <v>215</v>
+      </c>
+      <c r="B52" s="23" t="s">
+        <v>216</v>
+      </c>
+      <c r="C52" s="23" t="s">
+        <v>217</v>
+      </c>
+      <c r="D52" s="23" t="s">
+        <v>218</v>
+      </c>
+      <c r="E52" s="23" t="s">
+        <v>219</v>
+      </c>
+      <c r="F52" s="23" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="39" t="s">
+        <v>256</v>
+      </c>
+      <c r="B53" s="26" t="n">
+        <f aca="false">SUM(B5:B15)</f>
+        <v>100.67</v>
+      </c>
+      <c r="C53" s="26" t="n">
+        <f aca="false">SUM(C5:C15)</f>
+        <v>95.94</v>
+      </c>
+      <c r="D53" s="26" t="n">
+        <f aca="false">SUM(D5:D15)</f>
+        <v>95.16</v>
+      </c>
+      <c r="E53" s="26" t="n">
+        <f aca="false">SUM(E5:E15)</f>
+        <v>102.83</v>
+      </c>
+      <c r="F53" s="26" t="n">
+        <f aca="false">SUM(F5:F15)</f>
+        <v>100.27</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="39" t="s">
+        <v>257</v>
+      </c>
+      <c r="B54" s="26" t="n">
+        <f aca="false">B46*1.1792</f>
+        <v>9.598688</v>
+      </c>
+      <c r="C54" s="26" t="n">
+        <f aca="false">C46*1.1792</f>
+        <v>18.136096</v>
+      </c>
+      <c r="D54" s="26" t="n">
+        <f aca="false">D46*1.1792</f>
+        <v>9.068048</v>
+      </c>
+      <c r="E54" s="26" t="n">
+        <f aca="false">E46*1.1792</f>
+        <v>10.49488</v>
+      </c>
+      <c r="F54" s="26" t="n">
+        <f aca="false">F46*1.1792</f>
+        <v>10.25904</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="39" t="s">
+        <v>258</v>
+      </c>
+      <c r="B55" s="46" t="n">
+        <f aca="false">B44*1.1379</f>
+        <v>24.69243</v>
+      </c>
+      <c r="C55" s="46" t="n">
+        <f aca="false">C44*1.1379</f>
+        <v>35.38869</v>
+      </c>
+      <c r="D55" s="46" t="n">
+        <f aca="false">D44*1.1379</f>
+        <v>22.41663</v>
+      </c>
+      <c r="E55" s="46" t="n">
+        <f aca="false">E44*1.1379</f>
+        <v>36.18522</v>
+      </c>
+      <c r="F55" s="46" t="n">
+        <f aca="false">F44*1.1379</f>
+        <v>35.84385</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="39" t="s">
+        <v>259</v>
+      </c>
+      <c r="B56" s="26" t="n">
+        <f aca="false">B44/B46</f>
+        <v>2.66584766584767</v>
+      </c>
+      <c r="C56" s="26" t="n">
+        <f aca="false">C44/C46</f>
+        <v>2.0221066319896</v>
+      </c>
+      <c r="D56" s="26" t="n">
+        <f aca="false">D44/D46</f>
+        <v>2.56176853055917</v>
+      </c>
+      <c r="E56" s="26" t="n">
+        <f aca="false">E44/E46</f>
+        <v>3.57303370786517</v>
+      </c>
+      <c r="F56" s="26" t="n">
+        <f aca="false">F44/F46</f>
+        <v>3.62068965517241</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="39" t="s">
+        <v>260</v>
+      </c>
+      <c r="B57" s="26" t="n">
+        <f aca="false">(B11*2/61.98+B8*2/94.2)/(B5*2/101.96)</f>
+        <v>0.930733333650737</v>
+      </c>
+      <c r="C57" s="26" t="n">
+        <f aca="false">(C11*2/61.98+C8*2/94.2)/(C5*2/101.96)</f>
+        <v>0.759737054574487</v>
+      </c>
+      <c r="D57" s="26" t="n">
+        <f aca="false">(D11*2/61.98+D8*2/94.2)/(D5*2/101.96)</f>
+        <v>0.932786542456655</v>
+      </c>
+      <c r="E57" s="26" t="n">
+        <f aca="false">(E11*2/61.98+E8*2/94.2)/(E5*2/101.96)</f>
+        <v>0.903174143640449</v>
+      </c>
+      <c r="F57" s="26" t="n">
+        <f aca="false">(F11*2/61.98+F8*2/94.2)/(F5*2/101.96)</f>
+        <v>0.904643687235911</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="39" t="s">
+        <v>261</v>
+      </c>
+      <c r="B58" s="26" t="n">
+        <f aca="false">(B5*2/101.96)/(B6/56.08*2+B11*2/61.98+B8*2/94.2)</f>
+        <v>0.98213779934543</v>
+      </c>
+      <c r="C58" s="26" t="n">
+        <f aca="false">(C5*2/101.96)/(C6/56.08*2+C11*2/61.98+C8*2/94.2)</f>
+        <v>1.22744565834617</v>
+      </c>
+      <c r="D58" s="26" t="n">
+        <f aca="false">(D5*2/101.96)/(D6/56.08*2+D11*2/61.98+D8*2/94.2)</f>
+        <v>0.987371553214105</v>
+      </c>
+      <c r="E58" s="26" t="n">
+        <f aca="false">(E5*2/101.96)/(E6/56.08*2+E11*2/61.98+E8*2/94.2)</f>
+        <v>1.04079860572985</v>
+      </c>
+      <c r="F58" s="26" t="n">
+        <f aca="false">(F5*2/101.96)/(F6/56.08*2+F11*2/61.98+F8*2/94.2)</f>
+        <v>1.03239662662282</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="39" t="s">
+        <v>262</v>
+      </c>
+      <c r="B59" s="26" t="n">
+        <f aca="false">B28/(B5*0.5293)</f>
+        <v>5.86715517110809</v>
+      </c>
+      <c r="C59" s="26" t="n">
+        <f aca="false">C28/(C5*0.5293)</f>
+        <v>5.44090820481442</v>
+      </c>
+      <c r="D59" s="26" t="n">
+        <f aca="false">D28/(D5*0.5293)</f>
+        <v>5.86836571068272</v>
+      </c>
+      <c r="E59" s="26" t="n">
+        <f aca="false">E28/(E5*0.5293)</f>
+        <v>5.95829255096661</v>
+      </c>
+      <c r="F59" s="26" t="n">
+        <f aca="false">F28/(F5*0.5293)</f>
+        <v>6.0605629582721</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="39" t="s">
+        <v>263</v>
+      </c>
+      <c r="B60" s="25" t="n">
+        <f aca="false">B19+B35+B21+B48</f>
+        <v>636.37</v>
+      </c>
+      <c r="C60" s="25" t="n">
+        <f aca="false">C19+C35+C21+C48</f>
+        <v>587.73</v>
+      </c>
+      <c r="D60" s="25" t="n">
+        <f aca="false">D19+D35+D21+D48</f>
+        <v>655.39</v>
+      </c>
+      <c r="E60" s="25" t="n">
+        <f aca="false">E19+E35+E21+E48</f>
+        <v>594.87</v>
+      </c>
+      <c r="F60" s="25" t="n">
+        <f aca="false">F19+F35+F21+F48</f>
+        <v>593.15</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="39" t="s">
+        <v>264</v>
+      </c>
+      <c r="B61" s="25" t="n">
+        <f aca="false">B39/B17</f>
+        <v>23.65</v>
+      </c>
+      <c r="C61" s="25" t="n">
+        <f aca="false">C39/C17</f>
+        <v>21.6133333333333</v>
+      </c>
+      <c r="D61" s="25" t="n">
+        <f aca="false">D39/D17</f>
+        <v>23.5285714285714</v>
+      </c>
+      <c r="E61" s="25" t="n">
+        <f aca="false">E39/E17</f>
+        <v>38.28</v>
+      </c>
+      <c r="F61" s="25" t="n">
+        <f aca="false">F39/F17</f>
+        <v>37.15</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="39" t="s">
+        <v>265</v>
+      </c>
+      <c r="B62" s="49" t="n">
+        <f aca="false">IF(B27="","Eu&lt;LD",(B27/0.058)/SQRT((B40/0.153)*(B29/0.2055)))</f>
+        <v>0.00884232111570106</v>
+      </c>
+      <c r="C62" s="49" t="str">
+        <f aca="false">IF(C27="","Eu&lt;LD",(C27/0.058)/SQRT((C40/0.153)*(C29/0.2055)))</f>
+        <v>Eu&lt;LD</v>
+      </c>
+      <c r="D62" s="49" t="n">
+        <f aca="false">IF(D27="","Eu&lt;LD",(D27/0.058)/SQRT((D40/0.153)*(D29/0.2055)))</f>
+        <v>0.00866223878202</v>
+      </c>
+      <c r="E62" s="49" t="n">
+        <f aca="false">IF(E27="","Eu&lt;LD",(E27/0.058)/SQRT((E40/0.153)*(E29/0.2055)))</f>
+        <v>0.0109714044892516</v>
+      </c>
+      <c r="F62" s="49" t="n">
+        <f aca="false">IF(F27="","Eu&lt;LD",(F27/0.058)/SQRT((F40/0.153)*(F29/0.2055)))</f>
+        <v>0.0111695174796709</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="39" t="s">
+        <v>266</v>
+      </c>
+      <c r="B63" s="26" t="n">
+        <f aca="false">(B32/0.237)/(B49/0.17)</f>
+        <v>1.22078870496592</v>
+      </c>
+      <c r="C63" s="26" t="n">
+        <f aca="false">(C32/0.237)/(C49/0.17)</f>
+        <v>0.639914561339006</v>
+      </c>
+      <c r="D63" s="26" t="n">
+        <f aca="false">(D32/0.237)/(D49/0.17)</f>
+        <v>1.04955522677042</v>
+      </c>
+      <c r="E63" s="26" t="n">
+        <f aca="false">(E32/0.237)/(E49/0.17)</f>
+        <v>2.72022070756248</v>
+      </c>
+      <c r="F63" s="26" t="n">
+        <f aca="false">(F32/0.237)/(F49/0.17)</f>
+        <v>2.68711457319052</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="39" t="s">
+        <v>267</v>
+      </c>
+      <c r="B64" s="25" t="n">
+        <f aca="false">B46*12.35</f>
+        <v>100.529</v>
+      </c>
+      <c r="C64" s="25" t="n">
+        <f aca="false">C46*12.35</f>
+        <v>189.943</v>
+      </c>
+      <c r="D64" s="25" t="n">
+        <f aca="false">D46*12.35</f>
+        <v>94.9715</v>
+      </c>
+      <c r="E64" s="25" t="n">
+        <f aca="false">E46*12.35</f>
+        <v>109.915</v>
+      </c>
+      <c r="F64" s="25" t="n">
+        <f aca="false">F46*12.35</f>
+        <v>107.445</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="39" t="s">
+        <v>268</v>
+      </c>
+      <c r="B65" s="25" t="n">
+        <f aca="false">B44*4.06</f>
+        <v>88.102</v>
+      </c>
+      <c r="C65" s="25" t="n">
+        <f aca="false">C44*4.06</f>
+        <v>126.266</v>
+      </c>
+      <c r="D65" s="25" t="n">
+        <f aca="false">D44*4.06</f>
+        <v>79.982</v>
+      </c>
+      <c r="E65" s="25" t="n">
+        <f aca="false">E44*4.06</f>
+        <v>129.108</v>
+      </c>
+      <c r="F65" s="25" t="n">
+        <f aca="false">F44*4.06</f>
+        <v>127.89</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="39" t="s">
+        <v>269</v>
+      </c>
+      <c r="B66" s="25" t="n">
+        <f aca="false">B8*0.8301*313</f>
+        <v>1060.070904</v>
+      </c>
+      <c r="C66" s="25" t="n">
+        <f aca="false">C8*0.8301*313</f>
+        <v>937.954893</v>
+      </c>
+      <c r="D66" s="25" t="n">
+        <f aca="false">D8*0.8301*313</f>
+        <v>1039.2852</v>
+      </c>
+      <c r="E66" s="25" t="n">
+        <f aca="false">E8*0.8301*313</f>
+        <v>1132.820868</v>
+      </c>
+      <c r="F66" s="25" t="n">
+        <f aca="false">F8*0.8301*313</f>
+        <v>1093.847673</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="39" t="s">
+        <v>270</v>
+      </c>
+      <c r="B67" s="29" t="n">
+        <f aca="false">B64/300+B65/200+B66/3000</f>
+        <v>1.12896363466667</v>
+      </c>
+      <c r="C67" s="29" t="n">
+        <f aca="false">C64/300+C65/200+C66/3000</f>
+        <v>1.57712496433333</v>
+      </c>
+      <c r="D67" s="29" t="n">
+        <f aca="false">D64/300+D65/200+D66/3000</f>
+        <v>1.06291006666667</v>
+      </c>
+      <c r="E67" s="29" t="n">
+        <f aca="false">E64/300+E65/200+E66/3000</f>
+        <v>1.38953028933333</v>
+      </c>
+      <c r="F67" s="29" t="n">
+        <f aca="false">F64/300+F65/200+F66/3000</f>
+        <v>1.362215891</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="22" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="22" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="22" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="22" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="2" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="39" t="s">
+        <v>276</v>
+      </c>
+      <c r="B75" s="29" t="n">
+        <f aca="false">MEDIAN(B54:E54)</f>
+        <v>10.046784</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="39" t="s">
+        <v>277</v>
+      </c>
+      <c r="B76" s="29" t="n">
+        <f aca="false">Estatística!B6</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="39" t="s">
+        <v>278</v>
+      </c>
+      <c r="B77" s="29" t="str">
+        <f aca="false">TEXT(Estatística!B10,"0")&amp;"–"&amp;TEXT(Estatística!B13,"0")</f>
+        <v>5–12</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="39" t="s">
+        <v>279</v>
+      </c>
+      <c r="B78" s="29" t="str">
+        <f aca="false">TEXT(Estatística!C10,"0")&amp;"–"&amp;TEXT(Estatística!C13,"0")</f>
+        <v>4–26</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="39" t="s">
+        <v>280</v>
+      </c>
+      <c r="B79" s="29" t="n">
+        <f aca="false">Estatística!B52</f>
+        <v>20.1824816141584</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Adiciona aba de terras raras (TREO) e diagrama normalizado ao condrito
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017WeXEcDzNZfvUSeTFqUMWA
</commit_message>
<xml_diff>
--- a/uranio_diques_estatistica.xlsx
+++ b/uranio_diques_estatistica.xlsx
@@ -17,6 +17,7 @@
     <sheet name="Dendrograma" sheetId="7" state="visible" r:id="rId9"/>
     <sheet name="Comparação artigo" sheetId="8" state="visible" r:id="rId10"/>
     <sheet name="Laudo SGS 2024" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="ETR" sheetId="10" state="visible" r:id="rId12"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -50,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="316">
   <si>
     <t xml:space="preserve">Conclusões integradas (estatística das Tabelas 1–2 + matriz de correlação e dendrograma)</t>
   </si>
@@ -893,13 +894,118 @@
   </si>
   <si>
     <t xml:space="preserve">Limiar de anomalia do granito (média+2DP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Terras raras (ETR) – laudo SGS 2024, conversão para óxidos (TREO)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fatores elemento→óxido padrão (Ce como CeO2, Pr como Pr6O11, Tb como Tb4O7, demais R2O3). Teores em ppm; links em verde para a aba 'Laudo SGS 2024'.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fator óxido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La (óxido)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">leve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ce (óxido)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pr (óxido)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nd (óxido)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sm (óxido)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eu (óxido)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pesado+Y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gd (óxido)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tb (óxido)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dy (óxido)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ho (óxido)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Er (óxido)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tm (óxido)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yb (óxido)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lu (óxido)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Y (óxido)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TREO (ppm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TREO (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ETR pesados + Y (HREO) / TREO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Y2O3 / TREO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Óxidos 'ímã' Nd+Pr+Dy+Tb (ppm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dy2O3 + Tb4O7 (ppm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TREO / Th (quanto maior, menos radioativo por ETR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TREO relativo à crosta superior (~204 ppm TREO)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Referência: TREO da crosta continental superior (ppm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Soma dos ETR+Y de Rudnick &amp; Gao (2003) convertidos em óxidos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ordens de grandeza para comparação (aproximadas, variam por projeto):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Granito comum: ~150–300 ppm TREO.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Depósitos de argila iônica (regolito): tipicamente ~500–3.000 ppm TREO no horizonte enriquecido, com ETR extraíveis por troca iônica.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Depósitos em rocha dura (carbonatitos, pegmatitos, complexos alcalinos): em geral &gt; 1% TREO.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Os valores de 2024 são de rocha FRESCA (LOI ≤ 1,1%). O potencial para argila iônica depende do perfil de alteração, que não foi analisado.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="10">
+  <numFmts count="11">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
@@ -910,8 +1016,9 @@
     <numFmt numFmtId="171" formatCode="@"/>
     <numFmt numFmtId="172" formatCode="0.0"/>
     <numFmt numFmtId="173" formatCode="0.0\×"/>
+    <numFmt numFmtId="174" formatCode="0.000%"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1013,6 +1120,20 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF008000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="9"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -1095,7 +1216,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="56">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1296,6 +1417,30 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="172" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="174" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1452,6 +1597,48 @@
         <a:xfrm>
           <a:off x="0" y="571680"/>
           <a:ext cx="7286400" cy="5143320"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>176040</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>456840</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>80280</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11071080" y="571680"/>
+          <a:ext cx="7286400" cy="4285800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1748,6 +1935,672 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G36"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="0" width="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="22" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="23" t="s">
+        <v>158</v>
+      </c>
+      <c r="B4" s="23" t="s">
+        <v>283</v>
+      </c>
+      <c r="C4" s="23" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="23" t="s">
+        <v>216</v>
+      </c>
+      <c r="E4" s="23" t="s">
+        <v>217</v>
+      </c>
+      <c r="F4" s="23" t="s">
+        <v>218</v>
+      </c>
+      <c r="G4" s="23" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="24" t="s">
+        <v>284</v>
+      </c>
+      <c r="B5" s="43" t="n">
+        <v>1.1728</v>
+      </c>
+      <c r="C5" s="24" t="s">
+        <v>285</v>
+      </c>
+      <c r="D5" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!B32*$B5</f>
+        <v>41.51712</v>
+      </c>
+      <c r="E5" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!C32*$B5</f>
+        <v>25.2152</v>
+      </c>
+      <c r="F5" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!D32*$B5</f>
+        <v>39.64064</v>
+      </c>
+      <c r="G5" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!E32*$B5</f>
+        <v>57.81904</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="24" t="s">
+        <v>286</v>
+      </c>
+      <c r="B6" s="43" t="n">
+        <v>1.2284</v>
+      </c>
+      <c r="C6" s="24" t="s">
+        <v>285</v>
+      </c>
+      <c r="D6" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!B21*$B6</f>
+        <v>95.69236</v>
+      </c>
+      <c r="E6" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!C21*$B6</f>
+        <v>60.56012</v>
+      </c>
+      <c r="F6" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!D21*$B6</f>
+        <v>83.16268</v>
+      </c>
+      <c r="G6" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!E21*$B6</f>
+        <v>117.3122</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="24" t="s">
+        <v>287</v>
+      </c>
+      <c r="B7" s="43" t="n">
+        <v>1.2082</v>
+      </c>
+      <c r="C7" s="24" t="s">
+        <v>285</v>
+      </c>
+      <c r="D7" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!B38*$B7</f>
+        <v>11.888688</v>
+      </c>
+      <c r="E7" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!C38*$B7</f>
+        <v>7.8533</v>
+      </c>
+      <c r="F7" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!D38*$B7</f>
+        <v>10.257618</v>
+      </c>
+      <c r="G7" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!E38*$B7</f>
+        <v>14.969598</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="24" t="s">
+        <v>288</v>
+      </c>
+      <c r="B8" s="43" t="n">
+        <v>1.1664</v>
+      </c>
+      <c r="C8" s="24" t="s">
+        <v>285</v>
+      </c>
+      <c r="D8" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!B36*$B8</f>
+        <v>43.97328</v>
+      </c>
+      <c r="E8" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!C36*$B8</f>
+        <v>32.076</v>
+      </c>
+      <c r="F8" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!D36*$B8</f>
+        <v>39.30768</v>
+      </c>
+      <c r="G8" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!E36*$B8</f>
+        <v>53.88768</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="24" t="s">
+        <v>289</v>
+      </c>
+      <c r="B9" s="43" t="n">
+        <v>1.1596</v>
+      </c>
+      <c r="C9" s="24" t="s">
+        <v>285</v>
+      </c>
+      <c r="D9" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!B40*$B9</f>
+        <v>17.04612</v>
+      </c>
+      <c r="E9" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!C40*$B9</f>
+        <v>15.53864</v>
+      </c>
+      <c r="F9" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!D40*$B9</f>
+        <v>16.46632</v>
+      </c>
+      <c r="G9" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!E40*$B9</f>
+        <v>17.62592</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="24" t="s">
+        <v>290</v>
+      </c>
+      <c r="B10" s="43" t="n">
+        <v>1.1579</v>
+      </c>
+      <c r="C10" s="24" t="s">
+        <v>291</v>
+      </c>
+      <c r="D10" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!B27*$B10</f>
+        <v>0.057895</v>
+      </c>
+      <c r="E10" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!C27*$B10</f>
+        <v>0</v>
+      </c>
+      <c r="F10" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!D27*$B10</f>
+        <v>0.057895</v>
+      </c>
+      <c r="G10" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!E27*$B10</f>
+        <v>0.069474</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="24" t="s">
+        <v>292</v>
+      </c>
+      <c r="B11" s="43" t="n">
+        <v>1.1526</v>
+      </c>
+      <c r="C11" s="24" t="s">
+        <v>291</v>
+      </c>
+      <c r="D11" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!B29*$B11</f>
+        <v>23.432358</v>
+      </c>
+      <c r="E11" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!C29*$B11</f>
+        <v>26.440644</v>
+      </c>
+      <c r="F11" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!D29*$B11</f>
+        <v>25.276518</v>
+      </c>
+      <c r="G11" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!E29*$B11</f>
+        <v>21.196314</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="24" t="s">
+        <v>293</v>
+      </c>
+      <c r="B12" s="43" t="n">
+        <v>1.1762</v>
+      </c>
+      <c r="C12" s="24" t="s">
+        <v>291</v>
+      </c>
+      <c r="D12" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!B43*$B12</f>
+        <v>5.045898</v>
+      </c>
+      <c r="E12" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!C43*$B12</f>
+        <v>6.327956</v>
+      </c>
+      <c r="F12" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!D43*$B12</f>
+        <v>5.928048</v>
+      </c>
+      <c r="G12" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!E43*$B12</f>
+        <v>4.034366</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="24" t="s">
+        <v>294</v>
+      </c>
+      <c r="B13" s="43" t="n">
+        <v>1.1477</v>
+      </c>
+      <c r="C13" s="24" t="s">
+        <v>291</v>
+      </c>
+      <c r="D13" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!B25*$B13</f>
+        <v>36.818216</v>
+      </c>
+      <c r="E13" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!C25*$B13</f>
+        <v>49.052698</v>
+      </c>
+      <c r="F13" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!D25*$B13</f>
+        <v>45.047225</v>
+      </c>
+      <c r="G13" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!E25*$B13</f>
+        <v>26.224945</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="24" t="s">
+        <v>295</v>
+      </c>
+      <c r="B14" s="43" t="n">
+        <v>1.1455</v>
+      </c>
+      <c r="C14" s="24" t="s">
+        <v>291</v>
+      </c>
+      <c r="D14" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!B31*$B14</f>
+        <v>7.7894</v>
+      </c>
+      <c r="E14" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!C31*$B14</f>
+        <v>10.320955</v>
+      </c>
+      <c r="F14" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!D31*$B14</f>
+        <v>9.34728</v>
+      </c>
+      <c r="G14" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!E31*$B14</f>
+        <v>5.372395</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="24" t="s">
+        <v>296</v>
+      </c>
+      <c r="B15" s="43" t="n">
+        <v>1.1435</v>
+      </c>
+      <c r="C15" s="24" t="s">
+        <v>291</v>
+      </c>
+      <c r="D15" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!B26*$B15</f>
+        <v>25.11126</v>
+      </c>
+      <c r="E15" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!C26*$B15</f>
+        <v>32.646925</v>
+      </c>
+      <c r="F15" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!D26*$B15</f>
+        <v>29.673825</v>
+      </c>
+      <c r="G15" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!E26*$B15</f>
+        <v>16.10048</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="24" t="s">
+        <v>297</v>
+      </c>
+      <c r="B16" s="43" t="n">
+        <v>1.1421</v>
+      </c>
+      <c r="C16" s="24" t="s">
+        <v>291</v>
+      </c>
+      <c r="D16" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!B45*$B16</f>
+        <v>3.609036</v>
+      </c>
+      <c r="E16" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!C45*$B16</f>
+        <v>4.442769</v>
+      </c>
+      <c r="F16" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!D45*$B16</f>
+        <v>4.180086</v>
+      </c>
+      <c r="G16" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!E45*$B16</f>
+        <v>2.318463</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="24" t="s">
+        <v>298</v>
+      </c>
+      <c r="B17" s="43" t="n">
+        <v>1.1387</v>
+      </c>
+      <c r="C17" s="24" t="s">
+        <v>291</v>
+      </c>
+      <c r="D17" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!B49*$B17</f>
+        <v>23.68496</v>
+      </c>
+      <c r="E17" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!C49*$B17</f>
+        <v>27.44267</v>
+      </c>
+      <c r="F17" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!D49*$B17</f>
+        <v>26.30397</v>
+      </c>
+      <c r="G17" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!E49*$B17</f>
+        <v>14.8031</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="24" t="s">
+        <v>299</v>
+      </c>
+      <c r="B18" s="43" t="n">
+        <v>1.1371</v>
+      </c>
+      <c r="C18" s="24" t="s">
+        <v>291</v>
+      </c>
+      <c r="D18" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!B33*$B18</f>
+        <v>2.933718</v>
+      </c>
+      <c r="E18" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!C33*$B18</f>
+        <v>3.399929</v>
+      </c>
+      <c r="F18" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!D33*$B18</f>
+        <v>3.252106</v>
+      </c>
+      <c r="G18" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!E33*$B18</f>
+        <v>1.830731</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="24" t="s">
+        <v>300</v>
+      </c>
+      <c r="B19" s="43" t="n">
+        <v>1.2699</v>
+      </c>
+      <c r="C19" s="24" t="s">
+        <v>291</v>
+      </c>
+      <c r="D19" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!B48*$B19</f>
+        <v>255.808656</v>
+      </c>
+      <c r="E19" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!C48*$B19</f>
+        <v>329.145381</v>
+      </c>
+      <c r="F19" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!D48*$B19</f>
+        <v>321.03072</v>
+      </c>
+      <c r="G19" s="50" t="n">
+        <f aca="false">'Laudo SGS 2024'!E48*$B19</f>
+        <v>216.149679</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="D21" s="51" t="n">
+        <f aca="false">SUM(D5:D19)</f>
+        <v>594.408965</v>
+      </c>
+      <c r="E21" s="51" t="n">
+        <f aca="false">SUM(E5:E19)</f>
+        <v>630.463187</v>
+      </c>
+      <c r="F21" s="51" t="n">
+        <f aca="false">SUM(F5:F19)</f>
+        <v>658.932611</v>
+      </c>
+      <c r="G21" s="51" t="n">
+        <f aca="false">SUM(G5:G19)</f>
+        <v>569.714385</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="39" t="s">
+        <v>302</v>
+      </c>
+      <c r="D22" s="52" t="n">
+        <f aca="false">D21/10000</f>
+        <v>0.0594408965</v>
+      </c>
+      <c r="E22" s="52" t="n">
+        <f aca="false">E21/10000</f>
+        <v>0.0630463187</v>
+      </c>
+      <c r="F22" s="52" t="n">
+        <f aca="false">F21/10000</f>
+        <v>0.0658932611</v>
+      </c>
+      <c r="G22" s="52" t="n">
+        <f aca="false">G21/10000</f>
+        <v>0.0569714385</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="39" t="s">
+        <v>303</v>
+      </c>
+      <c r="D23" s="53" t="n">
+        <f aca="false">SUMIF($C$5:$C$19,"pesado+Y",D5:D19)/D21</f>
+        <v>0.646510095957251</v>
+      </c>
+      <c r="E23" s="53" t="n">
+        <f aca="false">SUMIF($C$5:$C$19,"pesado+Y",E5:E19)/E21</f>
+        <v>0.7759690606646</v>
+      </c>
+      <c r="F23" s="53" t="n">
+        <f aca="false">SUMIF($C$5:$C$19,"pesado+Y",F5:F19)/F21</f>
+        <v>0.71342298916816</v>
+      </c>
+      <c r="G23" s="53" t="n">
+        <f aca="false">SUMIF($C$5:$C$19,"pesado+Y",G5:G19)/G21</f>
+        <v>0.540797204901189</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="39" t="s">
+        <v>304</v>
+      </c>
+      <c r="D24" s="53" t="n">
+        <f aca="false">D19/D21</f>
+        <v>0.430358004442278</v>
+      </c>
+      <c r="E24" s="53" t="n">
+        <f aca="false">E19/E21</f>
+        <v>0.522069151358714</v>
+      </c>
+      <c r="F24" s="53" t="n">
+        <f aca="false">F19/F21</f>
+        <v>0.487198105907677</v>
+      </c>
+      <c r="G24" s="53" t="n">
+        <f aca="false">G19/G21</f>
+        <v>0.379400072546878</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="39" t="s">
+        <v>305</v>
+      </c>
+      <c r="D25" s="51" t="n">
+        <f aca="false">D8+D7+D13+D12</f>
+        <v>97.726082</v>
+      </c>
+      <c r="E25" s="51" t="n">
+        <f aca="false">E8+E7+E13+E12</f>
+        <v>95.309954</v>
+      </c>
+      <c r="F25" s="51" t="n">
+        <f aca="false">F8+F7+F13+F12</f>
+        <v>100.540571</v>
+      </c>
+      <c r="G25" s="51" t="n">
+        <f aca="false">G8+G7+G13+G12</f>
+        <v>99.116589</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="39" t="s">
+        <v>306</v>
+      </c>
+      <c r="D26" s="51" t="n">
+        <f aca="false">D13+D12</f>
+        <v>41.864114</v>
+      </c>
+      <c r="E26" s="51" t="n">
+        <f aca="false">E13+E12</f>
+        <v>55.380654</v>
+      </c>
+      <c r="F26" s="51" t="n">
+        <f aca="false">F13+F12</f>
+        <v>50.975273</v>
+      </c>
+      <c r="G26" s="51" t="n">
+        <f aca="false">G13+G12</f>
+        <v>30.259311</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="39" t="s">
+        <v>307</v>
+      </c>
+      <c r="D27" s="51" t="n">
+        <f aca="false">D21/'Laudo SGS 2024'!B44</f>
+        <v>27.392118202765</v>
+      </c>
+      <c r="E27" s="51" t="n">
+        <f aca="false">E21/'Laudo SGS 2024'!C44</f>
+        <v>20.2721281993569</v>
+      </c>
+      <c r="F27" s="51" t="n">
+        <f aca="false">F21/'Laudo SGS 2024'!D44</f>
+        <v>33.4483558883249</v>
+      </c>
+      <c r="G27" s="51" t="n">
+        <f aca="false">G21/'Laudo SGS 2024'!E44</f>
+        <v>17.9155466981132</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="39" t="s">
+        <v>308</v>
+      </c>
+      <c r="D28" s="54" t="n">
+        <f aca="false">D21/$B$30</f>
+        <v>2.91376943627451</v>
+      </c>
+      <c r="E28" s="54" t="n">
+        <f aca="false">E21/$B$30</f>
+        <v>3.09050581862745</v>
+      </c>
+      <c r="F28" s="54" t="n">
+        <f aca="false">F21/$B$30</f>
+        <v>3.23006181862745</v>
+      </c>
+      <c r="G28" s="54" t="n">
+        <f aca="false">G21/$B$30</f>
+        <v>2.79271757352941</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="39" t="s">
+        <v>309</v>
+      </c>
+      <c r="B30" s="31" t="n">
+        <v>204</v>
+      </c>
+      <c r="C30" s="22" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="55" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="22" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="22" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="22" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="22" t="s">
+        <v>315</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">

</xml_diff>